<commit_message>
TPS/TVQ, slide explanations, sounds, budget project, step-by-step notebook
- Practice lessons and Excel files now use Quebec taxes (TPS 5% + TVQ 9.975%)
- Slide decks with live, editable examples for all 17 practice lessons
- Project steps reveal one block at a time
- Soft UI sounds with a mute button
- New project: monthly budget
- Notebook entries gain "what you need", step-by-step guides and common mistakes
- Layout uses the screen better (quiz intro, practice, slides)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/calculateur-prix-depart-en.xlsx
+++ b/assets/calculateur-prix-depart-en.xlsx
@@ -37,16 +37,16 @@
     <t>Desired markup</t>
   </si>
   <si>
-    <t>VAT</t>
+    <t>Sales tax (GST + QST)</t>
   </si>
   <si>
     <t>Cost price</t>
   </si>
   <si>
-    <t>Selling price excl. VAT</t>
-  </si>
-  <si>
-    <t>Selling price incl. VAT</t>
+    <t>Selling price before tax</t>
+  </si>
+  <si>
+    <t>Selling price with tax</t>
   </si>
   <si>
     <t>Profit per product</t>
@@ -494,7 +494,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.2</v>
+        <v>0.14975</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>